<commit_message>
update before trial slides
</commit_message>
<xml_diff>
--- a/rec_long.xlsx
+++ b/rec_long.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Muhammad\Documents\Itzik\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{49FE1406-8FA5-4B46-8CD2-0FFF5F919C2F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E1E6092-EEED-4E2B-BB0A-6CE4D32FD9FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="7500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2588,33 +2588,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:IK31"/>
-  <sheetFormatPr defaultColWidth="5.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="5.68359375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" style="28" customWidth="1"/>
-    <col min="2" max="2" width="37.140625" style="28" customWidth="1"/>
-    <col min="3" max="23" width="5.7109375" style="28" customWidth="1"/>
-    <col min="24" max="24" width="14.42578125" style="28" customWidth="1"/>
-    <col min="25" max="25" width="23.42578125" style="28" customWidth="1"/>
-    <col min="26" max="26" width="14.42578125" style="28" customWidth="1"/>
-    <col min="27" max="61" width="5.7109375" style="28" customWidth="1"/>
-    <col min="62" max="62" width="12.28515625" style="28" customWidth="1"/>
-    <col min="63" max="97" width="5.7109375" style="28" customWidth="1"/>
-    <col min="98" max="98" width="15.7109375" style="28" customWidth="1"/>
-    <col min="99" max="99" width="23.42578125" style="28" customWidth="1"/>
-    <col min="100" max="100" width="15.7109375" style="28" customWidth="1"/>
-    <col min="101" max="135" width="5.7109375" style="28" customWidth="1"/>
-    <col min="136" max="136" width="9.28515625" style="28" customWidth="1"/>
-    <col min="137" max="171" width="5.7109375" style="28" customWidth="1"/>
+    <col min="1" max="1" width="18.578125" style="28" customWidth="1"/>
+    <col min="2" max="2" width="37.15625" style="28" customWidth="1"/>
+    <col min="3" max="23" width="5.68359375" style="28" customWidth="1"/>
+    <col min="24" max="24" width="14.41796875" style="28" customWidth="1"/>
+    <col min="25" max="25" width="23.41796875" style="28" customWidth="1"/>
+    <col min="26" max="26" width="14.41796875" style="28" customWidth="1"/>
+    <col min="27" max="61" width="5.68359375" style="28" customWidth="1"/>
+    <col min="62" max="62" width="12.26171875" style="28" customWidth="1"/>
+    <col min="63" max="97" width="5.68359375" style="28" customWidth="1"/>
+    <col min="98" max="98" width="15.68359375" style="28" customWidth="1"/>
+    <col min="99" max="99" width="23.41796875" style="28" customWidth="1"/>
+    <col min="100" max="100" width="15.68359375" style="28" customWidth="1"/>
+    <col min="101" max="135" width="5.68359375" style="28" customWidth="1"/>
+    <col min="136" max="136" width="9.26171875" style="28" customWidth="1"/>
+    <col min="137" max="171" width="5.68359375" style="28" customWidth="1"/>
     <col min="172" max="172" width="16" style="28" customWidth="1"/>
-    <col min="173" max="173" width="25.5703125" style="28" customWidth="1"/>
-    <col min="174" max="174" width="9.85546875" style="28" customWidth="1"/>
-    <col min="175" max="209" width="5.7109375" style="28" customWidth="1"/>
-    <col min="210" max="210" width="10.140625" style="28" customWidth="1"/>
-    <col min="211" max="213" width="5.7109375" style="28" customWidth="1"/>
-    <col min="214" max="16384" width="5.7109375" style="28"/>
+    <col min="173" max="173" width="25.578125" style="28" customWidth="1"/>
+    <col min="174" max="174" width="9.83984375" style="28" customWidth="1"/>
+    <col min="175" max="209" width="5.68359375" style="28" customWidth="1"/>
+    <col min="210" max="210" width="10.15625" style="28" customWidth="1"/>
+    <col min="211" max="213" width="5.68359375" style="28" customWidth="1"/>
+    <col min="214" max="16384" width="5.68359375" style="28"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:245" ht="14.45" customHeight="1">
+    <row r="1" spans="1:245" ht="14.5" customHeight="1">
       <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
@@ -3351,7 +3351,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="2" spans="1:245" ht="14.45" customHeight="1">
+    <row r="2" spans="1:245" ht="14.5" customHeight="1">
       <c r="A2" s="28" t="s">
         <v>80</v>
       </c>
@@ -3575,7 +3575,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:245" ht="14.45" customHeight="1">
+    <row r="3" spans="1:245" ht="14.5" customHeight="1">
       <c r="A3" s="28" t="s">
         <v>121</v>
       </c>
@@ -3799,7 +3799,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:245" ht="14.45" customHeight="1">
+    <row r="4" spans="1:245" ht="14.5" customHeight="1">
       <c r="A4" s="28" t="s">
         <v>123</v>
       </c>
@@ -4023,7 +4023,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:245" ht="14.45" customHeight="1">
+    <row r="5" spans="1:245" ht="14.5" customHeight="1">
       <c r="A5" s="28" t="s">
         <v>125</v>
       </c>
@@ -4247,7 +4247,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:245" ht="14.45" customHeight="1">
+    <row r="6" spans="1:245" ht="14.5" customHeight="1">
       <c r="A6" s="28" t="s">
         <v>126</v>
       </c>
@@ -4471,7 +4471,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:245" ht="14.45" customHeight="1">
+    <row r="7" spans="1:245" ht="14.5" customHeight="1">
       <c r="A7" s="28" t="s">
         <v>127</v>
       </c>
@@ -4695,7 +4695,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="1:245" ht="14.45" customHeight="1">
+    <row r="8" spans="1:245" ht="14.5" customHeight="1">
       <c r="A8" s="28" t="s">
         <v>128</v>
       </c>
@@ -4919,7 +4919,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:245" ht="14.45" customHeight="1">
+    <row r="9" spans="1:245" ht="14.5" customHeight="1">
       <c r="A9" s="28" t="s">
         <v>129</v>
       </c>
@@ -5143,7 +5143,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:245" ht="14.45" customHeight="1">
+    <row r="10" spans="1:245" ht="14.5" customHeight="1">
       <c r="A10" s="28" t="s">
         <v>130</v>
       </c>
@@ -5367,7 +5367,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:245" ht="14.45" customHeight="1">
+    <row r="11" spans="1:245" ht="14.5" customHeight="1">
       <c r="A11" s="28" t="s">
         <v>131</v>
       </c>
@@ -5591,7 +5591,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="12" spans="1:245" ht="14.45" customHeight="1">
+    <row r="12" spans="1:245" ht="14.5" customHeight="1">
       <c r="A12" s="28" t="s">
         <v>132</v>
       </c>
@@ -5815,7 +5815,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:245" ht="14.45" customHeight="1">
+    <row r="13" spans="1:245" ht="14.5" customHeight="1">
       <c r="A13" s="28" t="s">
         <v>160</v>
       </c>
@@ -6039,7 +6039,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:245" ht="14.45" customHeight="1">
+    <row r="14" spans="1:245" ht="14.5" customHeight="1">
       <c r="A14" s="28" t="s">
         <v>161</v>
       </c>
@@ -6263,7 +6263,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="15" spans="1:245" ht="14.45" customHeight="1">
+    <row r="15" spans="1:245" ht="14.5" customHeight="1">
       <c r="A15" s="28" t="s">
         <v>162</v>
       </c>
@@ -6487,7 +6487,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="16" spans="1:245" ht="14.45" customHeight="1">
+    <row r="16" spans="1:245" ht="14.5" customHeight="1">
       <c r="A16" s="28" t="s">
         <v>163</v>
       </c>
@@ -6711,7 +6711,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="1:80" ht="14.45" customHeight="1">
+    <row r="17" spans="1:80" ht="14.5" customHeight="1">
       <c r="A17" s="28" t="s">
         <v>164</v>
       </c>
@@ -6935,7 +6935,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:80" ht="14.45" customHeight="1">
+    <row r="18" spans="1:80" ht="14.5" customHeight="1">
       <c r="A18" s="28" t="s">
         <v>165</v>
       </c>
@@ -7159,7 +7159,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:80" ht="14.45" customHeight="1">
+    <row r="19" spans="1:80" ht="14.5" customHeight="1">
       <c r="A19" s="28" t="s">
         <v>166</v>
       </c>
@@ -7383,7 +7383,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="20" spans="1:80" ht="14.45" customHeight="1">
+    <row r="20" spans="1:80" ht="14.5" customHeight="1">
       <c r="A20" s="28" t="s">
         <v>167</v>
       </c>
@@ -7607,7 +7607,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:80" ht="14.45" customHeight="1">
+    <row r="21" spans="1:80" ht="14.5" customHeight="1">
       <c r="A21" s="28" t="s">
         <v>168</v>
       </c>
@@ -7831,7 +7831,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="22" spans="1:80" ht="14.45" customHeight="1">
+    <row r="22" spans="1:80" ht="14.5" customHeight="1">
       <c r="A22" s="28" t="s">
         <v>169</v>
       </c>
@@ -8055,7 +8055,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="23" spans="1:80" ht="14.45" customHeight="1">
+    <row r="23" spans="1:80" ht="14.5" customHeight="1">
       <c r="A23" s="28" t="s">
         <v>197</v>
       </c>
@@ -8279,7 +8279,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:80" ht="14.45" customHeight="1">
+    <row r="24" spans="1:80" ht="14.5" customHeight="1">
       <c r="A24" s="28" t="s">
         <v>198</v>
       </c>
@@ -8503,7 +8503,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:80" ht="14.45" customHeight="1">
+    <row r="25" spans="1:80" ht="14.5" customHeight="1">
       <c r="A25" s="28" t="s">
         <v>199</v>
       </c>
@@ -8727,7 +8727,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="26" spans="1:80" ht="14.45" customHeight="1">
+    <row r="26" spans="1:80" ht="14.5" customHeight="1">
       <c r="A26" s="28" t="s">
         <v>200</v>
       </c>
@@ -8951,7 +8951,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:80" ht="14.45" customHeight="1">
+    <row r="27" spans="1:80" ht="14.5" customHeight="1">
       <c r="A27" s="28" t="s">
         <v>201</v>
       </c>
@@ -9175,7 +9175,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="28" spans="1:80" ht="14.45" customHeight="1">
+    <row r="28" spans="1:80" ht="14.5" customHeight="1">
       <c r="A28" s="28" t="s">
         <v>202</v>
       </c>
@@ -9399,7 +9399,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:80" ht="14.45" customHeight="1">
+    <row r="29" spans="1:80" ht="14.5" customHeight="1">
       <c r="A29" s="28" t="s">
         <v>203</v>
       </c>
@@ -9623,7 +9623,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="30" spans="1:80" ht="14.45" customHeight="1">
+    <row r="30" spans="1:80" ht="14.5" customHeight="1">
       <c r="A30" s="28" t="s">
         <v>204</v>
       </c>
@@ -9847,7 +9847,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:80" ht="14.45" customHeight="1">
+    <row r="31" spans="1:80" ht="14.5" customHeight="1">
       <c r="A31" s="28" t="s">
         <v>205</v>
       </c>
@@ -10232,21 +10232,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:X31"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="5" width="13.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" style="1" customWidth="1"/>
-    <col min="10" max="18" width="7.42578125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="8.140625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="43.42578125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="9.140625" style="1" customWidth="1"/>
-    <col min="22" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="5" width="13.578125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="17.26171875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="13.15625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.41796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.41796875" style="1" customWidth="1"/>
+    <col min="10" max="18" width="7.41796875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="8.15625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="43.41796875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="9.15625" style="1" customWidth="1"/>
+    <col min="22" max="16384" width="9.15625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="14.45" customHeight="1">
+    <row r="1" spans="1:24" ht="14.5" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>206</v>
       </c>
@@ -12281,7 +12281,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I31"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16" style="26" customWidth="1"/>
     <col min="2" max="2" width="10" style="26" customWidth="1"/>
@@ -12292,7 +12292,7 @@
     <col min="9" max="9" width="11" style="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.45" customHeight="1">
+    <row r="1" spans="1:9" ht="14.5" customHeight="1">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -12321,7 +12321,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="28.5">
+    <row r="2" spans="1:9">
       <c r="A2" s="9" t="s">
         <v>80</v>
       </c>
@@ -12350,7 +12350,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="28.5">
+    <row r="3" spans="1:9">
       <c r="A3" s="9" t="s">
         <v>121</v>
       </c>
@@ -12379,7 +12379,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="28.5">
+    <row r="4" spans="1:9">
       <c r="A4" s="9" t="s">
         <v>123</v>
       </c>
@@ -12408,7 +12408,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="28.5">
+    <row r="5" spans="1:9">
       <c r="A5" s="9" t="s">
         <v>125</v>
       </c>
@@ -12437,7 +12437,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="28.5">
+    <row r="6" spans="1:9">
       <c r="A6" s="9" t="s">
         <v>126</v>
       </c>
@@ -12466,7 +12466,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="28.5">
+    <row r="7" spans="1:9">
       <c r="A7" s="9" t="s">
         <v>127</v>
       </c>
@@ -12495,7 +12495,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="28.5">
+    <row r="8" spans="1:9">
       <c r="A8" s="9" t="s">
         <v>128</v>
       </c>
@@ -12524,7 +12524,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="28.5">
+    <row r="9" spans="1:9">
       <c r="A9" s="9" t="s">
         <v>129</v>
       </c>
@@ -12553,7 +12553,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="28.5">
+    <row r="10" spans="1:9">
       <c r="A10" s="9" t="s">
         <v>130</v>
       </c>
@@ -12582,7 +12582,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="28.5">
+    <row r="11" spans="1:9">
       <c r="A11" s="9" t="s">
         <v>131</v>
       </c>
@@ -12611,7 +12611,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="28.5">
+    <row r="12" spans="1:9">
       <c r="A12" s="9" t="s">
         <v>132</v>
       </c>
@@ -12640,7 +12640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="28.5">
+    <row r="13" spans="1:9">
       <c r="A13" s="9" t="s">
         <v>160</v>
       </c>
@@ -12669,7 +12669,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="28.5">
+    <row r="14" spans="1:9">
       <c r="A14" s="9" t="s">
         <v>161</v>
       </c>
@@ -12698,7 +12698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="28.5">
+    <row r="15" spans="1:9">
       <c r="A15" s="9" t="s">
         <v>162</v>
       </c>
@@ -12727,7 +12727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="28.5">
+    <row r="16" spans="1:9">
       <c r="A16" s="9" t="s">
         <v>163</v>
       </c>
@@ -12756,7 +12756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="28.5">
+    <row r="17" spans="1:9">
       <c r="A17" s="9" t="s">
         <v>164</v>
       </c>
@@ -12785,7 +12785,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="28.5">
+    <row r="18" spans="1:9">
       <c r="A18" s="9" t="s">
         <v>165</v>
       </c>
@@ -12814,7 +12814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="28.5">
+    <row r="19" spans="1:9">
       <c r="A19" s="9" t="s">
         <v>166</v>
       </c>
@@ -12843,7 +12843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="28.5">
+    <row r="20" spans="1:9">
       <c r="A20" s="9" t="s">
         <v>167</v>
       </c>
@@ -12872,7 +12872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="28.5">
+    <row r="21" spans="1:9">
       <c r="A21" s="9" t="s">
         <v>168</v>
       </c>
@@ -12901,7 +12901,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="28.5">
+    <row r="22" spans="1:9">
       <c r="A22" s="9" t="s">
         <v>169</v>
       </c>
@@ -12930,7 +12930,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="28.5">
+    <row r="23" spans="1:9">
       <c r="A23" s="9" t="s">
         <v>197</v>
       </c>
@@ -12959,7 +12959,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="28.5">
+    <row r="24" spans="1:9">
       <c r="A24" s="9" t="s">
         <v>198</v>
       </c>
@@ -12988,7 +12988,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="28.5">
+    <row r="25" spans="1:9">
       <c r="A25" s="9" t="s">
         <v>199</v>
       </c>
@@ -13017,7 +13017,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="28.5">
+    <row r="26" spans="1:9">
       <c r="A26" s="9" t="s">
         <v>200</v>
       </c>
@@ -13046,7 +13046,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="28.5">
+    <row r="27" spans="1:9">
       <c r="A27" s="9" t="s">
         <v>201</v>
       </c>
@@ -13075,7 +13075,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="28.5">
+    <row r="28" spans="1:9">
       <c r="A28" s="9" t="s">
         <v>202</v>
       </c>
@@ -13104,7 +13104,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="28.5">
+    <row r="29" spans="1:9">
       <c r="A29" s="9" t="s">
         <v>203</v>
       </c>
@@ -13133,7 +13133,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="28.5">
+    <row r="30" spans="1:9">
       <c r="A30" s="9" t="s">
         <v>204</v>
       </c>
@@ -13162,7 +13162,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="28.5">
+    <row r="31" spans="1:9">
       <c r="A31" s="9" t="s">
         <v>205</v>
       </c>
@@ -13199,7 +13199,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:L901"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16" style="26" customWidth="1"/>
     <col min="2" max="2" width="10" style="26" customWidth="1"/>
@@ -13373,11 +13373,11 @@
       <c r="J5" s="12" t="s">
         <v>334</v>
       </c>
-      <c r="K5" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>232</v>
+      <c r="K5" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="30" customHeight="1">
@@ -13411,11 +13411,11 @@
       <c r="J6" s="12" t="s">
         <v>334</v>
       </c>
-      <c r="K6" s="9" t="s">
-        <v>244</v>
-      </c>
-      <c r="L6" s="9" t="s">
-        <v>244</v>
+      <c r="K6" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="L6" s="17" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="30" customHeight="1">
@@ -46740,7 +46740,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="21" style="26" customWidth="1"/>
     <col min="2" max="2" width="12" style="26" customWidth="1"/>
@@ -46758,7 +46758,7 @@
       <c r="D1" s="35"/>
       <c r="E1" s="35"/>
     </row>
-    <row r="3" spans="1:5" ht="14.45" customHeight="1">
+    <row r="3" spans="1:5" ht="14.5" customHeight="1">
       <c r="A3" s="25" t="s">
         <v>325</v>
       </c>
@@ -46814,7 +46814,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="14.45" customHeight="1">
+    <row r="8" spans="1:5" ht="14.5" customHeight="1">
       <c r="A8" s="25" t="s">
         <v>325</v>
       </c>

</xml_diff>